<commit_message>
fixed duplicate name in lunch checkoff, fixed missing person in lunch checkoff, and added outlook email drafts
</commit_message>
<xml_diff>
--- a/outputs/lunch_checkoff.xlsx
+++ b/outputs/lunch_checkoff.xlsx
@@ -721,11 +721,11 @@
         </is>
       </c>
       <c r="B17" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C17" s="8" t="inlineStr"/>
       <c r="D17" s="8" t="inlineStr"/>
-      <c r="E17" s="9" t="inlineStr"/>
+      <c r="E17" s="8" t="inlineStr"/>
       <c r="F17" s="9" t="inlineStr"/>
       <c r="G17" s="9" t="inlineStr"/>
     </row>
@@ -901,13 +901,13 @@
         </is>
       </c>
       <c r="B29" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C29" s="8" t="inlineStr"/>
       <c r="D29" s="8" t="inlineStr"/>
       <c r="E29" s="8" t="inlineStr"/>
       <c r="F29" s="8" t="inlineStr"/>
-      <c r="G29" s="8" t="inlineStr"/>
+      <c r="G29" s="9" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -1152,76 +1152,76 @@
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>Pedro Ovalle</t>
+          <t>Nirosha Sadinidhi Vijayan</t>
         </is>
       </c>
       <c r="B46" s="8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C46" s="8" t="inlineStr"/>
       <c r="D46" s="8" t="inlineStr"/>
-      <c r="E46" s="9" t="inlineStr"/>
-      <c r="F46" s="9" t="inlineStr"/>
+      <c r="E46" s="8" t="inlineStr"/>
+      <c r="F46" s="8" t="inlineStr"/>
       <c r="G46" s="9" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
         <is>
-          <t>Peikang Zhang</t>
+          <t>Pedro Ovalle</t>
         </is>
       </c>
       <c r="B47" s="8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C47" s="8" t="inlineStr"/>
       <c r="D47" s="8" t="inlineStr"/>
-      <c r="E47" s="8" t="inlineStr"/>
-      <c r="F47" s="8" t="inlineStr"/>
+      <c r="E47" s="9" t="inlineStr"/>
+      <c r="F47" s="9" t="inlineStr"/>
       <c r="G47" s="9" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>Phongchai Pengrai</t>
+          <t>Peikang Zhang</t>
         </is>
       </c>
       <c r="B48" s="8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C48" s="8" t="inlineStr"/>
       <c r="D48" s="8" t="inlineStr"/>
-      <c r="E48" s="9" t="inlineStr"/>
-      <c r="F48" s="9" t="inlineStr"/>
+      <c r="E48" s="8" t="inlineStr"/>
+      <c r="F48" s="8" t="inlineStr"/>
       <c r="G48" s="9" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
         <is>
-          <t>Poojitha Suraneni</t>
+          <t>Phongchai Pengrai</t>
         </is>
       </c>
       <c r="B49" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C49" s="8" t="inlineStr"/>
       <c r="D49" s="8" t="inlineStr"/>
-      <c r="E49" s="8" t="inlineStr"/>
+      <c r="E49" s="9" t="inlineStr"/>
       <c r="F49" s="9" t="inlineStr"/>
       <c r="G49" s="9" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>Prajwal Gowda</t>
+          <t>Poojitha Suraneni</t>
         </is>
       </c>
       <c r="B50" s="8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C50" s="8" t="inlineStr"/>
       <c r="D50" s="8" t="inlineStr"/>
       <c r="E50" s="8" t="inlineStr"/>
-      <c r="F50" s="8" t="inlineStr"/>
+      <c r="F50" s="9" t="inlineStr"/>
       <c r="G50" s="9" t="inlineStr"/>
     </row>
     <row r="51">

</xml_diff>

<commit_message>
Updated to be working on editing the quarterly drawings
</commit_message>
<xml_diff>
--- a/outputs/lunch_checkoff.xlsx
+++ b/outputs/lunch_checkoff.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="February Lunches" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="March Lunches" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G63"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -495,12 +495,12 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>February TRP lunches</t>
+          <t>March TRP lunches</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>ALL LUNCHES EXPIRE ON 03/31/2026</t>
+          <t>ALL LUNCHES EXPIRE ON 04/30/2026</t>
         </is>
       </c>
     </row>
@@ -556,12 +556,12 @@
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C6" s="8" t="inlineStr"/>
       <c r="D6" s="8" t="inlineStr"/>
-      <c r="E6" s="8" t="inlineStr"/>
-      <c r="F6" s="8" t="inlineStr"/>
+      <c r="E6" s="9" t="inlineStr"/>
+      <c r="F6" s="9" t="inlineStr"/>
       <c r="G6" s="9" t="inlineStr"/>
     </row>
     <row r="7">
@@ -571,10 +571,10 @@
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C7" s="8" t="inlineStr"/>
-      <c r="D7" s="8" t="inlineStr"/>
+      <c r="D7" s="9" t="inlineStr"/>
       <c r="E7" s="9" t="inlineStr"/>
       <c r="F7" s="9" t="inlineStr"/>
       <c r="G7" s="9" t="inlineStr"/>
@@ -586,93 +586,93 @@
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C8" s="8" t="inlineStr"/>
       <c r="D8" s="8" t="inlineStr"/>
-      <c r="E8" s="9" t="inlineStr"/>
+      <c r="E8" s="8" t="inlineStr"/>
       <c r="F8" s="9" t="inlineStr"/>
       <c r="G8" s="9" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>Amisha Patel</t>
+          <t>Alex Shearer</t>
         </is>
       </c>
       <c r="B9" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C9" s="8" t="inlineStr"/>
-      <c r="D9" s="8" t="inlineStr"/>
-      <c r="E9" s="8" t="inlineStr"/>
+      <c r="D9" s="9" t="inlineStr"/>
+      <c r="E9" s="9" t="inlineStr"/>
       <c r="F9" s="9" t="inlineStr"/>
       <c r="G9" s="9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Amit Rai</t>
+          <t>Amisha Patel</t>
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C10" s="8" t="inlineStr"/>
       <c r="D10" s="8" t="inlineStr"/>
       <c r="E10" s="8" t="inlineStr"/>
-      <c r="F10" s="8" t="inlineStr"/>
+      <c r="F10" s="9" t="inlineStr"/>
       <c r="G10" s="9" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>Anu Siriyal</t>
+          <t>Amit Rai</t>
         </is>
       </c>
       <c r="B11" s="8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C11" s="8" t="inlineStr"/>
-      <c r="D11" s="9" t="inlineStr"/>
-      <c r="E11" s="9" t="inlineStr"/>
-      <c r="F11" s="9" t="inlineStr"/>
+      <c r="D11" s="8" t="inlineStr"/>
+      <c r="E11" s="8" t="inlineStr"/>
+      <c r="F11" s="8" t="inlineStr"/>
       <c r="G11" s="9" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>Aravind Rameshan Thampi</t>
+          <t>Andy Lam</t>
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C12" s="8" t="inlineStr"/>
-      <c r="D12" s="8" t="inlineStr"/>
-      <c r="E12" s="8" t="inlineStr"/>
+      <c r="D12" s="9" t="inlineStr"/>
+      <c r="E12" s="9" t="inlineStr"/>
       <c r="F12" s="9" t="inlineStr"/>
       <c r="G12" s="9" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>Arun Kumar Padmanabhachari</t>
+          <t>Aravind Rameshan Thampi</t>
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C13" s="8" t="inlineStr"/>
       <c r="D13" s="8" t="inlineStr"/>
       <c r="E13" s="8" t="inlineStr"/>
-      <c r="F13" s="9" t="inlineStr"/>
+      <c r="F13" s="8" t="inlineStr"/>
       <c r="G13" s="9" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>Ashwini Kc</t>
+          <t>Arun Kumar Padmanabhachari</t>
         </is>
       </c>
       <c r="B14" s="8" t="n">
@@ -687,59 +687,59 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Atharva Lele</t>
+          <t>Ashwini Kc</t>
         </is>
       </c>
       <c r="B15" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C15" s="8" t="inlineStr"/>
       <c r="D15" s="8" t="inlineStr"/>
-      <c r="E15" s="9" t="inlineStr"/>
+      <c r="E15" s="8" t="inlineStr"/>
       <c r="F15" s="9" t="inlineStr"/>
       <c r="G15" s="9" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Athira Pillai</t>
+          <t>Atharva Lele</t>
         </is>
       </c>
       <c r="B16" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C16" s="8" t="inlineStr"/>
       <c r="D16" s="8" t="inlineStr"/>
-      <c r="E16" s="8" t="inlineStr"/>
+      <c r="E16" s="9" t="inlineStr"/>
       <c r="F16" s="9" t="inlineStr"/>
       <c r="G16" s="9" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>Calum Wilkie</t>
+          <t>Athira Pillai</t>
         </is>
       </c>
       <c r="B17" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C17" s="8" t="inlineStr"/>
       <c r="D17" s="8" t="inlineStr"/>
       <c r="E17" s="8" t="inlineStr"/>
-      <c r="F17" s="9" t="inlineStr"/>
+      <c r="F17" s="8" t="inlineStr"/>
       <c r="G17" s="9" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>Cecilia Pengrai</t>
+          <t>Attma Sharma</t>
         </is>
       </c>
       <c r="B18" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C18" s="8" t="inlineStr"/>
-      <c r="D18" s="8" t="inlineStr"/>
+      <c r="D18" s="9" t="inlineStr"/>
       <c r="E18" s="9" t="inlineStr"/>
       <c r="F18" s="9" t="inlineStr"/>
       <c r="G18" s="9" t="inlineStr"/>
@@ -747,122 +747,122 @@
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>Chakradhar Paladi</t>
+          <t>Calum Wilkie</t>
         </is>
       </c>
       <c r="B19" s="8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C19" s="8" t="inlineStr"/>
-      <c r="D19" s="9" t="inlineStr"/>
-      <c r="E19" s="9" t="inlineStr"/>
-      <c r="F19" s="9" t="inlineStr"/>
+      <c r="D19" s="8" t="inlineStr"/>
+      <c r="E19" s="8" t="inlineStr"/>
+      <c r="F19" s="8" t="inlineStr"/>
       <c r="G19" s="9" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>Chethan Raju</t>
+          <t>Cecilia Pengrai</t>
         </is>
       </c>
       <c r="B20" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C20" s="8" t="inlineStr"/>
-      <c r="D20" s="9" t="inlineStr"/>
-      <c r="E20" s="9" t="inlineStr"/>
+      <c r="D20" s="8" t="inlineStr"/>
+      <c r="E20" s="8" t="inlineStr"/>
       <c r="F20" s="9" t="inlineStr"/>
       <c r="G20" s="9" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>Christian Ramiscal</t>
+          <t>Chakradhar Paladi</t>
         </is>
       </c>
       <c r="B21" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C21" s="8" t="inlineStr"/>
       <c r="D21" s="8" t="inlineStr"/>
-      <c r="E21" s="8" t="inlineStr"/>
+      <c r="E21" s="9" t="inlineStr"/>
       <c r="F21" s="9" t="inlineStr"/>
       <c r="G21" s="9" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>Darshith Madvinkodi Prakash</t>
+          <t>Christian Ramiscal</t>
         </is>
       </c>
       <c r="B22" s="8" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C22" s="8" t="inlineStr"/>
-      <c r="D22" s="9" t="inlineStr"/>
-      <c r="E22" s="9" t="inlineStr"/>
-      <c r="F22" s="9" t="inlineStr"/>
-      <c r="G22" s="9" t="inlineStr"/>
+      <c r="D22" s="8" t="inlineStr"/>
+      <c r="E22" s="8" t="inlineStr"/>
+      <c r="F22" s="8" t="inlineStr"/>
+      <c r="G22" s="8" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>Edward Suh</t>
+          <t>Darshith Madvinkodi Prakash</t>
         </is>
       </c>
       <c r="B23" s="8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C23" s="8" t="inlineStr"/>
       <c r="D23" s="8" t="inlineStr"/>
       <c r="E23" s="8" t="inlineStr"/>
-      <c r="F23" s="8" t="inlineStr"/>
+      <c r="F23" s="9" t="inlineStr"/>
       <c r="G23" s="9" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>Emily Sheen</t>
+          <t>Edward Suh</t>
         </is>
       </c>
       <c r="B24" s="8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C24" s="8" t="inlineStr"/>
       <c r="D24" s="8" t="inlineStr"/>
-      <c r="E24" s="9" t="inlineStr"/>
-      <c r="F24" s="9" t="inlineStr"/>
-      <c r="G24" s="9" t="inlineStr"/>
+      <c r="E24" s="8" t="inlineStr"/>
+      <c r="F24" s="8" t="inlineStr"/>
+      <c r="G24" s="8" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>Ernesto Fajut</t>
+          <t>Emily Sheen</t>
         </is>
       </c>
       <c r="B25" s="8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C25" s="8" t="inlineStr"/>
       <c r="D25" s="8" t="inlineStr"/>
       <c r="E25" s="8" t="inlineStr"/>
-      <c r="F25" s="8" t="inlineStr"/>
+      <c r="F25" s="9" t="inlineStr"/>
       <c r="G25" s="9" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>Gabrielle Simms</t>
+          <t>Ernesto Fajut</t>
         </is>
       </c>
       <c r="B26" s="8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C26" s="8" t="inlineStr"/>
       <c r="D26" s="8" t="inlineStr"/>
-      <c r="E26" s="9" t="inlineStr"/>
-      <c r="F26" s="9" t="inlineStr"/>
-      <c r="G26" s="9" t="inlineStr"/>
+      <c r="E26" s="8" t="inlineStr"/>
+      <c r="F26" s="8" t="inlineStr"/>
+      <c r="G26" s="8" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -871,11 +871,11 @@
         </is>
       </c>
       <c r="B27" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C27" s="8" t="inlineStr"/>
       <c r="D27" s="8" t="inlineStr"/>
-      <c r="E27" s="9" t="inlineStr"/>
+      <c r="E27" s="8" t="inlineStr"/>
       <c r="F27" s="9" t="inlineStr"/>
       <c r="G27" s="9" t="inlineStr"/>
     </row>
@@ -886,48 +886,48 @@
         </is>
       </c>
       <c r="B28" s="8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C28" s="8" t="inlineStr"/>
       <c r="D28" s="8" t="inlineStr"/>
       <c r="E28" s="8" t="inlineStr"/>
       <c r="F28" s="8" t="inlineStr"/>
-      <c r="G28" s="9" t="inlineStr"/>
+      <c r="G28" s="8" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>Jennalyn Bayani</t>
+          <t>Jacky Lee</t>
         </is>
       </c>
       <c r="B29" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C29" s="8" t="inlineStr"/>
-      <c r="D29" s="8" t="inlineStr"/>
-      <c r="E29" s="8" t="inlineStr"/>
-      <c r="F29" s="8" t="inlineStr"/>
+      <c r="D29" s="9" t="inlineStr"/>
+      <c r="E29" s="9" t="inlineStr"/>
+      <c r="F29" s="9" t="inlineStr"/>
       <c r="G29" s="9" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>Jeremy John Patriarca</t>
+          <t>Jennalyn Bayani</t>
         </is>
       </c>
       <c r="B30" s="8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C30" s="8" t="inlineStr"/>
       <c r="D30" s="8" t="inlineStr"/>
       <c r="E30" s="8" t="inlineStr"/>
       <c r="F30" s="8" t="inlineStr"/>
-      <c r="G30" s="9" t="inlineStr"/>
+      <c r="G30" s="8" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>Jiajun Li</t>
+          <t>Jeremy John Patriarca</t>
         </is>
       </c>
       <c r="B31" s="8" t="n">
@@ -946,33 +946,33 @@
         </is>
       </c>
       <c r="B32" s="8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C32" s="8" t="inlineStr"/>
       <c r="D32" s="8" t="inlineStr"/>
-      <c r="E32" s="9" t="inlineStr"/>
-      <c r="F32" s="9" t="inlineStr"/>
+      <c r="E32" s="8" t="inlineStr"/>
+      <c r="F32" s="8" t="inlineStr"/>
       <c r="G32" s="9" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>John Bayani</t>
+          <t>Joe Walsh</t>
         </is>
       </c>
       <c r="B33" s="8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C33" s="8" t="inlineStr"/>
       <c r="D33" s="8" t="inlineStr"/>
       <c r="E33" s="8" t="inlineStr"/>
-      <c r="F33" s="8" t="inlineStr"/>
+      <c r="F33" s="9" t="inlineStr"/>
       <c r="G33" s="9" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>Johnson Jeffin George</t>
+          <t>John Bayani</t>
         </is>
       </c>
       <c r="B34" s="8" t="n">
@@ -987,7 +987,7 @@
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>Juan Rosales</t>
+          <t>Johnson Jeffin George</t>
         </is>
       </c>
       <c r="B35" s="8" t="n">
@@ -1002,31 +1002,31 @@
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>Kalp Patel</t>
+          <t>Juan Rosales</t>
         </is>
       </c>
       <c r="B36" s="8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C36" s="8" t="inlineStr"/>
       <c r="D36" s="8" t="inlineStr"/>
       <c r="E36" s="8" t="inlineStr"/>
       <c r="F36" s="8" t="inlineStr"/>
-      <c r="G36" s="9" t="inlineStr"/>
+      <c r="G36" s="8" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>Kashyap Meher</t>
+          <t>Kalp Patel</t>
         </is>
       </c>
       <c r="B37" s="8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C37" s="8" t="inlineStr"/>
       <c r="D37" s="8" t="inlineStr"/>
-      <c r="E37" s="9" t="inlineStr"/>
-      <c r="F37" s="9" t="inlineStr"/>
+      <c r="E37" s="8" t="inlineStr"/>
+      <c r="F37" s="8" t="inlineStr"/>
       <c r="G37" s="9" t="inlineStr"/>
     </row>
     <row r="38">
@@ -1036,10 +1036,10 @@
         </is>
       </c>
       <c r="B38" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C38" s="8" t="inlineStr"/>
-      <c r="D38" s="9" t="inlineStr"/>
+      <c r="D38" s="8" t="inlineStr"/>
       <c r="E38" s="9" t="inlineStr"/>
       <c r="F38" s="9" t="inlineStr"/>
       <c r="G38" s="9" t="inlineStr"/>
@@ -1062,7 +1062,7 @@
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>Margie R Isuga</t>
+          <t>Latchumanan Mathavan Murugappan</t>
         </is>
       </c>
       <c r="B40" s="8" t="n">
@@ -1077,7 +1077,7 @@
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
         <is>
-          <t>Michelle Tieu</t>
+          <t>Lucas Nelson</t>
         </is>
       </c>
       <c r="B41" s="8" t="n">
@@ -1092,7 +1092,7 @@
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>Midhun Mukundan Nair</t>
+          <t>Margie R Isuga</t>
         </is>
       </c>
       <c r="B42" s="8" t="n">
@@ -1107,7 +1107,7 @@
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>Mohit Sathyaseelan Palliyil</t>
+          <t>Michelle Tieu</t>
         </is>
       </c>
       <c r="B43" s="8" t="n">
@@ -1122,89 +1122,89 @@
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>Nandini Gajula</t>
+          <t>Midhun Mukundan Nair</t>
         </is>
       </c>
       <c r="B44" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C44" s="8" t="inlineStr"/>
-      <c r="D44" s="8" t="inlineStr"/>
-      <c r="E44" s="8" t="inlineStr"/>
+      <c r="D44" s="9" t="inlineStr"/>
+      <c r="E44" s="9" t="inlineStr"/>
       <c r="F44" s="9" t="inlineStr"/>
       <c r="G44" s="9" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>Naresh Tummalapalli</t>
+          <t>Midhun Mukundan Nair</t>
         </is>
       </c>
       <c r="B45" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C45" s="8" t="inlineStr"/>
       <c r="D45" s="8" t="inlineStr"/>
-      <c r="E45" s="8" t="inlineStr"/>
+      <c r="E45" s="9" t="inlineStr"/>
       <c r="F45" s="9" t="inlineStr"/>
       <c r="G45" s="9" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>Nirosha Sadinidhi Vijayan</t>
+          <t>Mohit Sathyaseelan Palliyil</t>
         </is>
       </c>
       <c r="B46" s="8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C46" s="8" t="inlineStr"/>
       <c r="D46" s="8" t="inlineStr"/>
       <c r="E46" s="8" t="inlineStr"/>
-      <c r="F46" s="8" t="inlineStr"/>
+      <c r="F46" s="9" t="inlineStr"/>
       <c r="G46" s="9" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
         <is>
-          <t>Pedro Ovalle</t>
+          <t>Nandini Gajula</t>
         </is>
       </c>
       <c r="B47" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C47" s="8" t="inlineStr"/>
       <c r="D47" s="8" t="inlineStr"/>
-      <c r="E47" s="9" t="inlineStr"/>
+      <c r="E47" s="8" t="inlineStr"/>
       <c r="F47" s="9" t="inlineStr"/>
       <c r="G47" s="9" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>Peikang Zhang</t>
+          <t>Naresh Tummalapalli</t>
         </is>
       </c>
       <c r="B48" s="8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C48" s="8" t="inlineStr"/>
       <c r="D48" s="8" t="inlineStr"/>
-      <c r="E48" s="8" t="inlineStr"/>
-      <c r="F48" s="8" t="inlineStr"/>
+      <c r="E48" s="9" t="inlineStr"/>
+      <c r="F48" s="9" t="inlineStr"/>
       <c r="G48" s="9" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
         <is>
-          <t>Phongchai Pengrai</t>
+          <t>Nilesh Rajbharti</t>
         </is>
       </c>
       <c r="B49" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C49" s="8" t="inlineStr"/>
-      <c r="D49" s="8" t="inlineStr"/>
+      <c r="D49" s="9" t="inlineStr"/>
       <c r="E49" s="9" t="inlineStr"/>
       <c r="F49" s="9" t="inlineStr"/>
       <c r="G49" s="9" t="inlineStr"/>
@@ -1212,52 +1212,52 @@
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>Poojitha Suraneni</t>
+          <t>Nirosha Sadinidhi Vijayan</t>
         </is>
       </c>
       <c r="B50" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C50" s="8" t="inlineStr"/>
       <c r="D50" s="8" t="inlineStr"/>
       <c r="E50" s="8" t="inlineStr"/>
-      <c r="F50" s="9" t="inlineStr"/>
+      <c r="F50" s="8" t="inlineStr"/>
       <c r="G50" s="9" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>Prajwal Gowda</t>
+          <t>Nithyasri Nara</t>
         </is>
       </c>
       <c r="B51" s="8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C51" s="8" t="inlineStr"/>
       <c r="D51" s="8" t="inlineStr"/>
-      <c r="E51" s="8" t="inlineStr"/>
-      <c r="F51" s="8" t="inlineStr"/>
+      <c r="E51" s="9" t="inlineStr"/>
+      <c r="F51" s="9" t="inlineStr"/>
       <c r="G51" s="9" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>Rahol Saha</t>
+          <t>Pedro Ovalle</t>
         </is>
       </c>
       <c r="B52" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C52" s="8" t="inlineStr"/>
-      <c r="D52" s="9" t="inlineStr"/>
-      <c r="E52" s="9" t="inlineStr"/>
+      <c r="D52" s="8" t="inlineStr"/>
+      <c r="E52" s="8" t="inlineStr"/>
       <c r="F52" s="9" t="inlineStr"/>
       <c r="G52" s="9" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>Rob Mcintosh</t>
+          <t>Peikang Zhang</t>
         </is>
       </c>
       <c r="B53" s="8" t="n">
@@ -1272,74 +1272,74 @@
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>Rohan Nayak</t>
+          <t>Phongchai Pengrai</t>
         </is>
       </c>
       <c r="B54" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C54" s="8" t="inlineStr"/>
       <c r="D54" s="8" t="inlineStr"/>
-      <c r="E54" s="9" t="inlineStr"/>
+      <c r="E54" s="8" t="inlineStr"/>
       <c r="F54" s="9" t="inlineStr"/>
       <c r="G54" s="9" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
         <is>
-          <t>Samir Fuke</t>
+          <t>Poojitha Suraneni</t>
         </is>
       </c>
       <c r="B55" s="8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C55" s="8" t="inlineStr"/>
       <c r="D55" s="8" t="inlineStr"/>
       <c r="E55" s="8" t="inlineStr"/>
-      <c r="F55" s="8" t="inlineStr"/>
+      <c r="F55" s="9" t="inlineStr"/>
       <c r="G55" s="9" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>Sathya Induri</t>
+          <t>Prajwal Gowda</t>
         </is>
       </c>
       <c r="B56" s="8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C56" s="8" t="inlineStr"/>
-      <c r="D56" s="9" t="inlineStr"/>
-      <c r="E56" s="9" t="inlineStr"/>
-      <c r="F56" s="9" t="inlineStr"/>
+      <c r="D56" s="8" t="inlineStr"/>
+      <c r="E56" s="8" t="inlineStr"/>
+      <c r="F56" s="8" t="inlineStr"/>
       <c r="G56" s="9" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
         <is>
-          <t>Shivani Palkar</t>
+          <t>Rahol Saha</t>
         </is>
       </c>
       <c r="B57" s="8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C57" s="8" t="inlineStr"/>
-      <c r="D57" s="9" t="inlineStr"/>
-      <c r="E57" s="9" t="inlineStr"/>
-      <c r="F57" s="9" t="inlineStr"/>
+      <c r="D57" s="8" t="inlineStr"/>
+      <c r="E57" s="8" t="inlineStr"/>
+      <c r="F57" s="8" t="inlineStr"/>
       <c r="G57" s="9" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>Sidhartha Gorajala</t>
+          <t>Rob Mcintosh</t>
         </is>
       </c>
       <c r="B58" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C58" s="8" t="inlineStr"/>
-      <c r="D58" s="8" t="inlineStr"/>
+      <c r="D58" s="9" t="inlineStr"/>
       <c r="E58" s="9" t="inlineStr"/>
       <c r="F58" s="9" t="inlineStr"/>
       <c r="G58" s="9" t="inlineStr"/>
@@ -1347,7 +1347,7 @@
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
         <is>
-          <t>Srividya Gopala Reddy</t>
+          <t>Rohan Nayak</t>
         </is>
       </c>
       <c r="B59" s="8" t="n">
@@ -1362,7 +1362,7 @@
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>Tony Lam</t>
+          <t>Samir Fuke</t>
         </is>
       </c>
       <c r="B60" s="8" t="n">
@@ -1377,7 +1377,7 @@
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
-          <t>Trayson Rubio</t>
+          <t>Sathya Induri</t>
         </is>
       </c>
       <c r="B61" s="8" t="n">
@@ -1392,32 +1392,137 @@
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>Varadparesh Keni</t>
+          <t>Sathya Induri</t>
         </is>
       </c>
       <c r="B62" s="8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C62" s="8" t="inlineStr"/>
-      <c r="D62" s="8" t="inlineStr"/>
-      <c r="E62" s="8" t="inlineStr"/>
-      <c r="F62" s="8" t="inlineStr"/>
-      <c r="G62" s="8" t="inlineStr"/>
+      <c r="D62" s="9" t="inlineStr"/>
+      <c r="E62" s="9" t="inlineStr"/>
+      <c r="F62" s="9" t="inlineStr"/>
+      <c r="G62" s="9" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
         <is>
-          <t>Yuga Pasupulate</t>
+          <t>Shivani Palkar</t>
         </is>
       </c>
       <c r="B63" s="8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C63" s="8" t="inlineStr"/>
       <c r="D63" s="8" t="inlineStr"/>
-      <c r="E63" s="8" t="inlineStr"/>
-      <c r="F63" s="8" t="inlineStr"/>
+      <c r="E63" s="9" t="inlineStr"/>
+      <c r="F63" s="9" t="inlineStr"/>
       <c r="G63" s="9" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="7" t="inlineStr">
+        <is>
+          <t>Sidhartha Gorajala</t>
+        </is>
+      </c>
+      <c r="B64" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C64" s="8" t="inlineStr"/>
+      <c r="D64" s="8" t="inlineStr"/>
+      <c r="E64" s="8" t="inlineStr"/>
+      <c r="F64" s="9" t="inlineStr"/>
+      <c r="G64" s="9" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="7" t="inlineStr">
+        <is>
+          <t>Srividya Gopala Reddy</t>
+        </is>
+      </c>
+      <c r="B65" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C65" s="8" t="inlineStr"/>
+      <c r="D65" s="8" t="inlineStr"/>
+      <c r="E65" s="9" t="inlineStr"/>
+      <c r="F65" s="9" t="inlineStr"/>
+      <c r="G65" s="9" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="7" t="inlineStr">
+        <is>
+          <t>Tony Lam</t>
+        </is>
+      </c>
+      <c r="B66" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="C66" s="8" t="inlineStr"/>
+      <c r="D66" s="8" t="inlineStr"/>
+      <c r="E66" s="8" t="inlineStr"/>
+      <c r="F66" s="8" t="inlineStr"/>
+      <c r="G66" s="8" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="7" t="inlineStr">
+        <is>
+          <t>Trayson Rubio</t>
+        </is>
+      </c>
+      <c r="B67" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C67" s="8" t="inlineStr"/>
+      <c r="D67" s="9" t="inlineStr"/>
+      <c r="E67" s="9" t="inlineStr"/>
+      <c r="F67" s="9" t="inlineStr"/>
+      <c r="G67" s="9" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="7" t="inlineStr">
+        <is>
+          <t>Varadparesh Keni</t>
+        </is>
+      </c>
+      <c r="B68" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="C68" s="8" t="inlineStr"/>
+      <c r="D68" s="8" t="inlineStr"/>
+      <c r="E68" s="8" t="inlineStr"/>
+      <c r="F68" s="8" t="inlineStr"/>
+      <c r="G68" s="8" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="7" t="inlineStr">
+        <is>
+          <t>Vincent Abraham</t>
+        </is>
+      </c>
+      <c r="B69" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="C69" s="8" t="inlineStr"/>
+      <c r="D69" s="8" t="inlineStr"/>
+      <c r="E69" s="8" t="inlineStr"/>
+      <c r="F69" s="8" t="inlineStr"/>
+      <c r="G69" s="9" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="7" t="inlineStr">
+        <is>
+          <t>Yuga Pasupulate</t>
+        </is>
+      </c>
+      <c r="B70" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="C70" s="8" t="inlineStr"/>
+      <c r="D70" s="8" t="inlineStr"/>
+      <c r="E70" s="8" t="inlineStr"/>
+      <c r="F70" s="8" t="inlineStr"/>
+      <c r="G70" s="9" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
oops now it is ready lol
</commit_message>
<xml_diff>
--- a/outputs/lunch_checkoff.xlsx
+++ b/outputs/lunch_checkoff.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -556,10 +556,10 @@
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C6" s="8" t="inlineStr"/>
-      <c r="D6" s="8" t="inlineStr"/>
+      <c r="D6" s="9" t="inlineStr"/>
       <c r="E6" s="9" t="inlineStr"/>
       <c r="F6" s="9" t="inlineStr"/>
       <c r="G6" s="9" t="inlineStr"/>
@@ -646,10 +646,10 @@
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C12" s="8" t="inlineStr"/>
-      <c r="D12" s="9" t="inlineStr"/>
+      <c r="D12" s="8" t="inlineStr"/>
       <c r="E12" s="9" t="inlineStr"/>
       <c r="F12" s="9" t="inlineStr"/>
       <c r="G12" s="9" t="inlineStr"/>
@@ -676,11 +676,11 @@
         </is>
       </c>
       <c r="B14" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C14" s="8" t="inlineStr"/>
       <c r="D14" s="8" t="inlineStr"/>
-      <c r="E14" s="9" t="inlineStr"/>
+      <c r="E14" s="8" t="inlineStr"/>
       <c r="F14" s="9" t="inlineStr"/>
       <c r="G14" s="9" t="inlineStr"/>
     </row>
@@ -867,127 +867,127 @@
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>Glenn Detruz</t>
+          <t>Gabrielle Simms</t>
         </is>
       </c>
       <c r="B27" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C27" s="8" t="inlineStr"/>
-      <c r="D27" s="8" t="inlineStr"/>
-      <c r="E27" s="8" t="inlineStr"/>
+      <c r="D27" s="9" t="inlineStr"/>
+      <c r="E27" s="9" t="inlineStr"/>
       <c r="F27" s="9" t="inlineStr"/>
       <c r="G27" s="9" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>Grace Fajut</t>
+          <t>Glenn Detruz</t>
         </is>
       </c>
       <c r="B28" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C28" s="8" t="inlineStr"/>
       <c r="D28" s="8" t="inlineStr"/>
       <c r="E28" s="8" t="inlineStr"/>
       <c r="F28" s="8" t="inlineStr"/>
-      <c r="G28" s="8" t="inlineStr"/>
+      <c r="G28" s="9" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>Jacky Lee</t>
+          <t>Grace Fajut</t>
         </is>
       </c>
       <c r="B29" s="8" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C29" s="8" t="inlineStr"/>
-      <c r="D29" s="9" t="inlineStr"/>
-      <c r="E29" s="9" t="inlineStr"/>
-      <c r="F29" s="9" t="inlineStr"/>
-      <c r="G29" s="9" t="inlineStr"/>
+      <c r="D29" s="8" t="inlineStr"/>
+      <c r="E29" s="8" t="inlineStr"/>
+      <c r="F29" s="8" t="inlineStr"/>
+      <c r="G29" s="8" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>Jennalyn Bayani</t>
+          <t>Jacky Lee</t>
         </is>
       </c>
       <c r="B30" s="8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C30" s="8" t="inlineStr"/>
-      <c r="D30" s="8" t="inlineStr"/>
-      <c r="E30" s="8" t="inlineStr"/>
-      <c r="F30" s="8" t="inlineStr"/>
-      <c r="G30" s="8" t="inlineStr"/>
+      <c r="D30" s="9" t="inlineStr"/>
+      <c r="E30" s="9" t="inlineStr"/>
+      <c r="F30" s="9" t="inlineStr"/>
+      <c r="G30" s="9" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>Jeremy John Patriarca</t>
+          <t>Jennalyn Bayani</t>
         </is>
       </c>
       <c r="B31" s="8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C31" s="8" t="inlineStr"/>
       <c r="D31" s="8" t="inlineStr"/>
-      <c r="E31" s="9" t="inlineStr"/>
-      <c r="F31" s="9" t="inlineStr"/>
-      <c r="G31" s="9" t="inlineStr"/>
+      <c r="E31" s="8" t="inlineStr"/>
+      <c r="F31" s="8" t="inlineStr"/>
+      <c r="G31" s="8" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>Jihan Huang</t>
+          <t>Jeremy John Patriarca</t>
         </is>
       </c>
       <c r="B32" s="8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C32" s="8" t="inlineStr"/>
       <c r="D32" s="8" t="inlineStr"/>
-      <c r="E32" s="8" t="inlineStr"/>
-      <c r="F32" s="8" t="inlineStr"/>
+      <c r="E32" s="9" t="inlineStr"/>
+      <c r="F32" s="9" t="inlineStr"/>
       <c r="G32" s="9" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>Joe Walsh</t>
+          <t>Jihan Huang</t>
         </is>
       </c>
       <c r="B33" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C33" s="8" t="inlineStr"/>
       <c r="D33" s="8" t="inlineStr"/>
       <c r="E33" s="8" t="inlineStr"/>
-      <c r="F33" s="9" t="inlineStr"/>
+      <c r="F33" s="8" t="inlineStr"/>
       <c r="G33" s="9" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>John Bayani</t>
+          <t>Joe Walsh</t>
         </is>
       </c>
       <c r="B34" s="8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C34" s="8" t="inlineStr"/>
       <c r="D34" s="8" t="inlineStr"/>
       <c r="E34" s="8" t="inlineStr"/>
-      <c r="F34" s="8" t="inlineStr"/>
+      <c r="F34" s="9" t="inlineStr"/>
       <c r="G34" s="9" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>Johnson Jeffin George</t>
+          <t>John Bayani</t>
         </is>
       </c>
       <c r="B35" s="8" t="n">
@@ -1002,59 +1002,59 @@
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>Juan Rosales</t>
+          <t>Johnson Jeffin George</t>
         </is>
       </c>
       <c r="B36" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C36" s="8" t="inlineStr"/>
       <c r="D36" s="8" t="inlineStr"/>
       <c r="E36" s="8" t="inlineStr"/>
       <c r="F36" s="8" t="inlineStr"/>
-      <c r="G36" s="8" t="inlineStr"/>
+      <c r="G36" s="9" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>Kalp Patel</t>
+          <t>Juan Rosales</t>
         </is>
       </c>
       <c r="B37" s="8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C37" s="8" t="inlineStr"/>
       <c r="D37" s="8" t="inlineStr"/>
       <c r="E37" s="8" t="inlineStr"/>
       <c r="F37" s="8" t="inlineStr"/>
-      <c r="G37" s="9" t="inlineStr"/>
+      <c r="G37" s="8" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>Kathie Ton</t>
+          <t>Kalp Patel</t>
         </is>
       </c>
       <c r="B38" s="8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C38" s="8" t="inlineStr"/>
       <c r="D38" s="8" t="inlineStr"/>
-      <c r="E38" s="9" t="inlineStr"/>
-      <c r="F38" s="9" t="inlineStr"/>
+      <c r="E38" s="8" t="inlineStr"/>
+      <c r="F38" s="8" t="inlineStr"/>
       <c r="G38" s="9" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
         <is>
-          <t>Kati Shackelford</t>
+          <t>Kathie Ton</t>
         </is>
       </c>
       <c r="B39" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C39" s="8" t="inlineStr"/>
-      <c r="D39" s="9" t="inlineStr"/>
+      <c r="D39" s="8" t="inlineStr"/>
       <c r="E39" s="9" t="inlineStr"/>
       <c r="F39" s="9" t="inlineStr"/>
       <c r="G39" s="9" t="inlineStr"/>
@@ -1062,74 +1062,74 @@
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>Latchumanan Mathavan Murugappan</t>
+          <t>Kati Shackelford</t>
         </is>
       </c>
       <c r="B40" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C40" s="8" t="inlineStr"/>
-      <c r="D40" s="8" t="inlineStr"/>
-      <c r="E40" s="8" t="inlineStr"/>
-      <c r="F40" s="8" t="inlineStr"/>
+      <c r="D40" s="9" t="inlineStr"/>
+      <c r="E40" s="9" t="inlineStr"/>
+      <c r="F40" s="9" t="inlineStr"/>
       <c r="G40" s="9" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
         <is>
-          <t>Lucas Nelson</t>
+          <t>Latchumanan Mathavan Murugappan</t>
         </is>
       </c>
       <c r="B41" s="8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C41" s="8" t="inlineStr"/>
-      <c r="D41" s="9" t="inlineStr"/>
-      <c r="E41" s="9" t="inlineStr"/>
-      <c r="F41" s="9" t="inlineStr"/>
+      <c r="D41" s="8" t="inlineStr"/>
+      <c r="E41" s="8" t="inlineStr"/>
+      <c r="F41" s="8" t="inlineStr"/>
       <c r="G41" s="9" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>Margie R Isuga</t>
+          <t>Lucas Nelson</t>
         </is>
       </c>
       <c r="B42" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C42" s="8" t="inlineStr"/>
-      <c r="D42" s="8" t="inlineStr"/>
-      <c r="E42" s="8" t="inlineStr"/>
-      <c r="F42" s="8" t="inlineStr"/>
+      <c r="D42" s="9" t="inlineStr"/>
+      <c r="E42" s="9" t="inlineStr"/>
+      <c r="F42" s="9" t="inlineStr"/>
       <c r="G42" s="9" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>Michelle Tieu</t>
+          <t>Margie R Isuga</t>
         </is>
       </c>
       <c r="B43" s="8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C43" s="8" t="inlineStr"/>
       <c r="D43" s="8" t="inlineStr"/>
-      <c r="E43" s="9" t="inlineStr"/>
-      <c r="F43" s="9" t="inlineStr"/>
+      <c r="E43" s="8" t="inlineStr"/>
+      <c r="F43" s="8" t="inlineStr"/>
       <c r="G43" s="9" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>Midhun Mukundan Nair</t>
+          <t>Michelle Tieu</t>
         </is>
       </c>
       <c r="B44" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C44" s="8" t="inlineStr"/>
-      <c r="D44" s="9" t="inlineStr"/>
+      <c r="D44" s="8" t="inlineStr"/>
       <c r="E44" s="9" t="inlineStr"/>
       <c r="F44" s="9" t="inlineStr"/>
       <c r="G44" s="9" t="inlineStr"/>
@@ -1141,12 +1141,12 @@
         </is>
       </c>
       <c r="B45" s="8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C45" s="8" t="inlineStr"/>
       <c r="D45" s="8" t="inlineStr"/>
-      <c r="E45" s="9" t="inlineStr"/>
-      <c r="F45" s="9" t="inlineStr"/>
+      <c r="E45" s="8" t="inlineStr"/>
+      <c r="F45" s="8" t="inlineStr"/>
       <c r="G45" s="9" t="inlineStr"/>
     </row>
     <row r="46">
@@ -1381,10 +1381,10 @@
         </is>
       </c>
       <c r="B61" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C61" s="8" t="inlineStr"/>
-      <c r="D61" s="9" t="inlineStr"/>
+      <c r="D61" s="8" t="inlineStr"/>
       <c r="E61" s="9" t="inlineStr"/>
       <c r="F61" s="9" t="inlineStr"/>
       <c r="G61" s="9" t="inlineStr"/>
@@ -1392,14 +1392,14 @@
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>Sathya Induri</t>
+          <t>Shivani Palkar</t>
         </is>
       </c>
       <c r="B62" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C62" s="8" t="inlineStr"/>
-      <c r="D62" s="9" t="inlineStr"/>
+      <c r="D62" s="8" t="inlineStr"/>
       <c r="E62" s="9" t="inlineStr"/>
       <c r="F62" s="9" t="inlineStr"/>
       <c r="G62" s="9" t="inlineStr"/>
@@ -1407,97 +1407,97 @@
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
         <is>
-          <t>Shivani Palkar</t>
+          <t>Sidhartha Gorajala</t>
         </is>
       </c>
       <c r="B63" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C63" s="8" t="inlineStr"/>
       <c r="D63" s="8" t="inlineStr"/>
-      <c r="E63" s="9" t="inlineStr"/>
+      <c r="E63" s="8" t="inlineStr"/>
       <c r="F63" s="9" t="inlineStr"/>
       <c r="G63" s="9" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
         <is>
-          <t>Sidhartha Gorajala</t>
+          <t>Srividya Gopala Reddy</t>
         </is>
       </c>
       <c r="B64" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C64" s="8" t="inlineStr"/>
       <c r="D64" s="8" t="inlineStr"/>
-      <c r="E64" s="8" t="inlineStr"/>
+      <c r="E64" s="9" t="inlineStr"/>
       <c r="F64" s="9" t="inlineStr"/>
       <c r="G64" s="9" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
         <is>
-          <t>Srividya Gopala Reddy</t>
+          <t>Tony Lam</t>
         </is>
       </c>
       <c r="B65" s="8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C65" s="8" t="inlineStr"/>
       <c r="D65" s="8" t="inlineStr"/>
-      <c r="E65" s="9" t="inlineStr"/>
-      <c r="F65" s="9" t="inlineStr"/>
+      <c r="E65" s="8" t="inlineStr"/>
+      <c r="F65" s="8" t="inlineStr"/>
       <c r="G65" s="9" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
         <is>
-          <t>Tony Lam</t>
+          <t>Trayson Rubio</t>
         </is>
       </c>
       <c r="B66" s="8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C66" s="8" t="inlineStr"/>
-      <c r="D66" s="8" t="inlineStr"/>
-      <c r="E66" s="8" t="inlineStr"/>
-      <c r="F66" s="8" t="inlineStr"/>
-      <c r="G66" s="8" t="inlineStr"/>
+      <c r="D66" s="9" t="inlineStr"/>
+      <c r="E66" s="9" t="inlineStr"/>
+      <c r="F66" s="9" t="inlineStr"/>
+      <c r="G66" s="9" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
         <is>
-          <t>Trayson Rubio</t>
+          <t>Varadparesh Keni</t>
         </is>
       </c>
       <c r="B67" s="8" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C67" s="8" t="inlineStr"/>
-      <c r="D67" s="9" t="inlineStr"/>
-      <c r="E67" s="9" t="inlineStr"/>
-      <c r="F67" s="9" t="inlineStr"/>
-      <c r="G67" s="9" t="inlineStr"/>
+      <c r="D67" s="8" t="inlineStr"/>
+      <c r="E67" s="8" t="inlineStr"/>
+      <c r="F67" s="8" t="inlineStr"/>
+      <c r="G67" s="8" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
         <is>
-          <t>Varadparesh Keni</t>
+          <t>Vincent Abraham</t>
         </is>
       </c>
       <c r="B68" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C68" s="8" t="inlineStr"/>
       <c r="D68" s="8" t="inlineStr"/>
       <c r="E68" s="8" t="inlineStr"/>
       <c r="F68" s="8" t="inlineStr"/>
-      <c r="G68" s="8" t="inlineStr"/>
+      <c r="G68" s="9" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
         <is>
-          <t>Vincent Abraham</t>
+          <t>Yuga Pasupulate</t>
         </is>
       </c>
       <c r="B69" s="8" t="n">
@@ -1508,21 +1508,6 @@
       <c r="E69" s="8" t="inlineStr"/>
       <c r="F69" s="8" t="inlineStr"/>
       <c r="G69" s="9" t="inlineStr"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="7" t="inlineStr">
-        <is>
-          <t>Yuga Pasupulate</t>
-        </is>
-      </c>
-      <c r="B70" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="C70" s="8" t="inlineStr"/>
-      <c r="D70" s="8" t="inlineStr"/>
-      <c r="E70" s="8" t="inlineStr"/>
-      <c r="F70" s="8" t="inlineStr"/>
-      <c r="G70" s="9" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
trying to commit codex changes so it audits that people dont try to get two trips out of one date
</commit_message>
<xml_diff>
--- a/outputs/lunch_checkoff.xlsx
+++ b/outputs/lunch_checkoff.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="March Lunches" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="April Lunches" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G69"/>
+  <dimension ref="A1:G65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -495,12 +495,12 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>March TRP lunches</t>
+          <t>April TRP lunches</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>ALL LUNCHES EXPIRE ON 04/30/2026</t>
+          <t>ALL LUNCHES EXPIRE ON 05/31/2026</t>
         </is>
       </c>
     </row>
@@ -556,12 +556,12 @@
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C6" s="8" t="inlineStr"/>
-      <c r="D6" s="9" t="inlineStr"/>
-      <c r="E6" s="9" t="inlineStr"/>
-      <c r="F6" s="9" t="inlineStr"/>
+      <c r="D6" s="8" t="inlineStr"/>
+      <c r="E6" s="8" t="inlineStr"/>
+      <c r="F6" s="8" t="inlineStr"/>
       <c r="G6" s="9" t="inlineStr"/>
     </row>
     <row r="7">
@@ -571,10 +571,10 @@
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7" s="8" t="inlineStr"/>
-      <c r="D7" s="9" t="inlineStr"/>
+      <c r="D7" s="8" t="inlineStr"/>
       <c r="E7" s="9" t="inlineStr"/>
       <c r="F7" s="9" t="inlineStr"/>
       <c r="G7" s="9" t="inlineStr"/>
@@ -586,11 +586,11 @@
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C8" s="8" t="inlineStr"/>
-      <c r="D8" s="8" t="inlineStr"/>
-      <c r="E8" s="8" t="inlineStr"/>
+      <c r="D8" s="9" t="inlineStr"/>
+      <c r="E8" s="9" t="inlineStr"/>
       <c r="F8" s="9" t="inlineStr"/>
       <c r="G8" s="9" t="inlineStr"/>
     </row>
@@ -616,11 +616,11 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C10" s="8" t="inlineStr"/>
       <c r="D10" s="8" t="inlineStr"/>
-      <c r="E10" s="8" t="inlineStr"/>
+      <c r="E10" s="9" t="inlineStr"/>
       <c r="F10" s="9" t="inlineStr"/>
       <c r="G10" s="9" t="inlineStr"/>
     </row>
@@ -676,12 +676,12 @@
         </is>
       </c>
       <c r="B14" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C14" s="8" t="inlineStr"/>
       <c r="D14" s="8" t="inlineStr"/>
       <c r="E14" s="8" t="inlineStr"/>
-      <c r="F14" s="9" t="inlineStr"/>
+      <c r="F14" s="8" t="inlineStr"/>
       <c r="G14" s="9" t="inlineStr"/>
     </row>
     <row r="15">
@@ -706,10 +706,10 @@
         </is>
       </c>
       <c r="B16" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C16" s="8" t="inlineStr"/>
-      <c r="D16" s="8" t="inlineStr"/>
+      <c r="D16" s="9" t="inlineStr"/>
       <c r="E16" s="9" t="inlineStr"/>
       <c r="F16" s="9" t="inlineStr"/>
       <c r="G16" s="9" t="inlineStr"/>
@@ -751,12 +751,12 @@
         </is>
       </c>
       <c r="B19" s="8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C19" s="8" t="inlineStr"/>
       <c r="D19" s="8" t="inlineStr"/>
       <c r="E19" s="8" t="inlineStr"/>
-      <c r="F19" s="8" t="inlineStr"/>
+      <c r="F19" s="9" t="inlineStr"/>
       <c r="G19" s="9" t="inlineStr"/>
     </row>
     <row r="20">
@@ -766,11 +766,11 @@
         </is>
       </c>
       <c r="B20" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C20" s="8" t="inlineStr"/>
-      <c r="D20" s="8" t="inlineStr"/>
-      <c r="E20" s="8" t="inlineStr"/>
+      <c r="D20" s="9" t="inlineStr"/>
+      <c r="E20" s="9" t="inlineStr"/>
       <c r="F20" s="9" t="inlineStr"/>
       <c r="G20" s="9" t="inlineStr"/>
     </row>
@@ -781,10 +781,10 @@
         </is>
       </c>
       <c r="B21" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C21" s="8" t="inlineStr"/>
-      <c r="D21" s="8" t="inlineStr"/>
+      <c r="D21" s="9" t="inlineStr"/>
       <c r="E21" s="9" t="inlineStr"/>
       <c r="F21" s="9" t="inlineStr"/>
       <c r="G21" s="9" t="inlineStr"/>
@@ -796,13 +796,13 @@
         </is>
       </c>
       <c r="B22" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C22" s="8" t="inlineStr"/>
       <c r="D22" s="8" t="inlineStr"/>
       <c r="E22" s="8" t="inlineStr"/>
       <c r="F22" s="8" t="inlineStr"/>
-      <c r="G22" s="8" t="inlineStr"/>
+      <c r="G22" s="9" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -841,11 +841,11 @@
         </is>
       </c>
       <c r="B25" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C25" s="8" t="inlineStr"/>
       <c r="D25" s="8" t="inlineStr"/>
-      <c r="E25" s="8" t="inlineStr"/>
+      <c r="E25" s="9" t="inlineStr"/>
       <c r="F25" s="9" t="inlineStr"/>
       <c r="G25" s="9" t="inlineStr"/>
     </row>
@@ -856,13 +856,13 @@
         </is>
       </c>
       <c r="B26" s="8" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C26" s="8" t="inlineStr"/>
       <c r="D26" s="8" t="inlineStr"/>
       <c r="E26" s="8" t="inlineStr"/>
-      <c r="F26" s="8" t="inlineStr"/>
-      <c r="G26" s="8" t="inlineStr"/>
+      <c r="F26" s="9" t="inlineStr"/>
+      <c r="G26" s="9" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -886,12 +886,12 @@
         </is>
       </c>
       <c r="B28" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C28" s="8" t="inlineStr"/>
-      <c r="D28" s="8" t="inlineStr"/>
-      <c r="E28" s="8" t="inlineStr"/>
-      <c r="F28" s="8" t="inlineStr"/>
+      <c r="D28" s="9" t="inlineStr"/>
+      <c r="E28" s="9" t="inlineStr"/>
+      <c r="F28" s="9" t="inlineStr"/>
       <c r="G28" s="9" t="inlineStr"/>
     </row>
     <row r="29">
@@ -901,13 +901,13 @@
         </is>
       </c>
       <c r="B29" s="8" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C29" s="8" t="inlineStr"/>
       <c r="D29" s="8" t="inlineStr"/>
       <c r="E29" s="8" t="inlineStr"/>
-      <c r="F29" s="8" t="inlineStr"/>
-      <c r="G29" s="8" t="inlineStr"/>
+      <c r="F29" s="9" t="inlineStr"/>
+      <c r="G29" s="9" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -916,10 +916,10 @@
         </is>
       </c>
       <c r="B30" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C30" s="8" t="inlineStr"/>
-      <c r="D30" s="9" t="inlineStr"/>
+      <c r="D30" s="8" t="inlineStr"/>
       <c r="E30" s="9" t="inlineStr"/>
       <c r="F30" s="9" t="inlineStr"/>
       <c r="G30" s="9" t="inlineStr"/>
@@ -942,22 +942,22 @@
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>Jeremy John Patriarca</t>
+          <t>Jennifer Goslin</t>
         </is>
       </c>
       <c r="B32" s="8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C32" s="8" t="inlineStr"/>
       <c r="D32" s="8" t="inlineStr"/>
-      <c r="E32" s="9" t="inlineStr"/>
-      <c r="F32" s="9" t="inlineStr"/>
+      <c r="E32" s="8" t="inlineStr"/>
+      <c r="F32" s="8" t="inlineStr"/>
       <c r="G32" s="9" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>Jihan Huang</t>
+          <t>Jeremy John Patriarca</t>
         </is>
       </c>
       <c r="B33" s="8" t="n">
@@ -976,12 +976,12 @@
         </is>
       </c>
       <c r="B34" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C34" s="8" t="inlineStr"/>
       <c r="D34" s="8" t="inlineStr"/>
       <c r="E34" s="8" t="inlineStr"/>
-      <c r="F34" s="9" t="inlineStr"/>
+      <c r="F34" s="8" t="inlineStr"/>
       <c r="G34" s="9" t="inlineStr"/>
     </row>
     <row r="35">
@@ -991,13 +991,13 @@
         </is>
       </c>
       <c r="B35" s="8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C35" s="8" t="inlineStr"/>
       <c r="D35" s="8" t="inlineStr"/>
       <c r="E35" s="8" t="inlineStr"/>
       <c r="F35" s="8" t="inlineStr"/>
-      <c r="G35" s="9" t="inlineStr"/>
+      <c r="G35" s="8" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -1006,12 +1006,12 @@
         </is>
       </c>
       <c r="B36" s="8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C36" s="8" t="inlineStr"/>
       <c r="D36" s="8" t="inlineStr"/>
-      <c r="E36" s="8" t="inlineStr"/>
-      <c r="F36" s="8" t="inlineStr"/>
+      <c r="E36" s="9" t="inlineStr"/>
+      <c r="F36" s="9" t="inlineStr"/>
       <c r="G36" s="9" t="inlineStr"/>
     </row>
     <row r="37">
@@ -1021,13 +1021,13 @@
         </is>
       </c>
       <c r="B37" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C37" s="8" t="inlineStr"/>
       <c r="D37" s="8" t="inlineStr"/>
       <c r="E37" s="8" t="inlineStr"/>
       <c r="F37" s="8" t="inlineStr"/>
-      <c r="G37" s="8" t="inlineStr"/>
+      <c r="G37" s="9" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -1036,18 +1036,18 @@
         </is>
       </c>
       <c r="B38" s="8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C38" s="8" t="inlineStr"/>
       <c r="D38" s="8" t="inlineStr"/>
-      <c r="E38" s="8" t="inlineStr"/>
-      <c r="F38" s="8" t="inlineStr"/>
+      <c r="E38" s="9" t="inlineStr"/>
+      <c r="F38" s="9" t="inlineStr"/>
       <c r="G38" s="9" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
         <is>
-          <t>Kathie Ton</t>
+          <t>Kashyap Meher</t>
         </is>
       </c>
       <c r="B39" s="8" t="n">
@@ -1096,11 +1096,11 @@
         </is>
       </c>
       <c r="B42" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C42" s="8" t="inlineStr"/>
-      <c r="D42" s="9" t="inlineStr"/>
-      <c r="E42" s="9" t="inlineStr"/>
+      <c r="D42" s="8" t="inlineStr"/>
+      <c r="E42" s="8" t="inlineStr"/>
       <c r="F42" s="9" t="inlineStr"/>
       <c r="G42" s="9" t="inlineStr"/>
     </row>
@@ -1122,37 +1122,37 @@
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>Michelle Tieu</t>
+          <t>Midhun Mukundan Nair</t>
         </is>
       </c>
       <c r="B44" s="8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C44" s="8" t="inlineStr"/>
       <c r="D44" s="8" t="inlineStr"/>
-      <c r="E44" s="9" t="inlineStr"/>
-      <c r="F44" s="9" t="inlineStr"/>
+      <c r="E44" s="8" t="inlineStr"/>
+      <c r="F44" s="8" t="inlineStr"/>
       <c r="G44" s="9" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>Midhun Mukundan Nair</t>
+          <t>Mohit Sathyaseelan Palliyil</t>
         </is>
       </c>
       <c r="B45" s="8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C45" s="8" t="inlineStr"/>
       <c r="D45" s="8" t="inlineStr"/>
-      <c r="E45" s="8" t="inlineStr"/>
-      <c r="F45" s="8" t="inlineStr"/>
+      <c r="E45" s="9" t="inlineStr"/>
+      <c r="F45" s="9" t="inlineStr"/>
       <c r="G45" s="9" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>Mohit Sathyaseelan Palliyil</t>
+          <t>Nandini Gajula</t>
         </is>
       </c>
       <c r="B46" s="8" t="n">
@@ -1167,7 +1167,7 @@
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
         <is>
-          <t>Nandini Gajula</t>
+          <t>Naresh Tummalapalli</t>
         </is>
       </c>
       <c r="B47" s="8" t="n">
@@ -1182,7 +1182,7 @@
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>Naresh Tummalapalli</t>
+          <t>Nilesh Rajbharti</t>
         </is>
       </c>
       <c r="B48" s="8" t="n">
@@ -1197,37 +1197,37 @@
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
         <is>
-          <t>Nilesh Rajbharti</t>
+          <t>Nirosha Sadinidhi Vijayan</t>
         </is>
       </c>
       <c r="B49" s="8" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C49" s="8" t="inlineStr"/>
-      <c r="D49" s="9" t="inlineStr"/>
-      <c r="E49" s="9" t="inlineStr"/>
-      <c r="F49" s="9" t="inlineStr"/>
-      <c r="G49" s="9" t="inlineStr"/>
+      <c r="D49" s="8" t="inlineStr"/>
+      <c r="E49" s="8" t="inlineStr"/>
+      <c r="F49" s="8" t="inlineStr"/>
+      <c r="G49" s="8" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>Nirosha Sadinidhi Vijayan</t>
+          <t>Nithyasri Nara</t>
         </is>
       </c>
       <c r="B50" s="8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C50" s="8" t="inlineStr"/>
       <c r="D50" s="8" t="inlineStr"/>
       <c r="E50" s="8" t="inlineStr"/>
-      <c r="F50" s="8" t="inlineStr"/>
+      <c r="F50" s="9" t="inlineStr"/>
       <c r="G50" s="9" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>Nithyasri Nara</t>
+          <t>Pedro Ovalle</t>
         </is>
       </c>
       <c r="B51" s="8" t="n">
@@ -1242,22 +1242,22 @@
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>Pedro Ovalle</t>
+          <t>Phongchai Pengrai</t>
         </is>
       </c>
       <c r="B52" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C52" s="8" t="inlineStr"/>
-      <c r="D52" s="8" t="inlineStr"/>
-      <c r="E52" s="8" t="inlineStr"/>
+      <c r="D52" s="9" t="inlineStr"/>
+      <c r="E52" s="9" t="inlineStr"/>
       <c r="F52" s="9" t="inlineStr"/>
       <c r="G52" s="9" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>Peikang Zhang</t>
+          <t>Poojitha Suraneni</t>
         </is>
       </c>
       <c r="B53" s="8" t="n">
@@ -1272,67 +1272,67 @@
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>Phongchai Pengrai</t>
+          <t>Prajwal Gowda</t>
         </is>
       </c>
       <c r="B54" s="8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C54" s="8" t="inlineStr"/>
       <c r="D54" s="8" t="inlineStr"/>
       <c r="E54" s="8" t="inlineStr"/>
-      <c r="F54" s="9" t="inlineStr"/>
-      <c r="G54" s="9" t="inlineStr"/>
+      <c r="F54" s="8" t="inlineStr"/>
+      <c r="G54" s="8" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
         <is>
-          <t>Poojitha Suraneni</t>
+          <t>Rahol Saha</t>
         </is>
       </c>
       <c r="B55" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C55" s="8" t="inlineStr"/>
       <c r="D55" s="8" t="inlineStr"/>
       <c r="E55" s="8" t="inlineStr"/>
-      <c r="F55" s="9" t="inlineStr"/>
+      <c r="F55" s="8" t="inlineStr"/>
       <c r="G55" s="9" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>Prajwal Gowda</t>
+          <t>Rob Mcintosh</t>
         </is>
       </c>
       <c r="B56" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C56" s="8" t="inlineStr"/>
-      <c r="D56" s="8" t="inlineStr"/>
-      <c r="E56" s="8" t="inlineStr"/>
-      <c r="F56" s="8" t="inlineStr"/>
+      <c r="D56" s="9" t="inlineStr"/>
+      <c r="E56" s="9" t="inlineStr"/>
+      <c r="F56" s="9" t="inlineStr"/>
       <c r="G56" s="9" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
         <is>
-          <t>Rahol Saha</t>
+          <t>Rohan Nayak</t>
         </is>
       </c>
       <c r="B57" s="8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C57" s="8" t="inlineStr"/>
       <c r="D57" s="8" t="inlineStr"/>
-      <c r="E57" s="8" t="inlineStr"/>
-      <c r="F57" s="8" t="inlineStr"/>
+      <c r="E57" s="9" t="inlineStr"/>
+      <c r="F57" s="9" t="inlineStr"/>
       <c r="G57" s="9" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>Rob Mcintosh</t>
+          <t>Shivani Palkar</t>
         </is>
       </c>
       <c r="B58" s="8" t="n">
@@ -1347,14 +1347,14 @@
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
         <is>
-          <t>Rohan Nayak</t>
+          <t>Sidhartha Gorajala</t>
         </is>
       </c>
       <c r="B59" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C59" s="8" t="inlineStr"/>
-      <c r="D59" s="9" t="inlineStr"/>
+      <c r="D59" s="8" t="inlineStr"/>
       <c r="E59" s="9" t="inlineStr"/>
       <c r="F59" s="9" t="inlineStr"/>
       <c r="G59" s="9" t="inlineStr"/>
@@ -1362,152 +1362,92 @@
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>Samir Fuke</t>
+          <t>Srividya Gopala Reddy</t>
         </is>
       </c>
       <c r="B60" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C60" s="8" t="inlineStr"/>
-      <c r="D60" s="8" t="inlineStr"/>
-      <c r="E60" s="8" t="inlineStr"/>
-      <c r="F60" s="8" t="inlineStr"/>
+      <c r="D60" s="9" t="inlineStr"/>
+      <c r="E60" s="9" t="inlineStr"/>
+      <c r="F60" s="9" t="inlineStr"/>
       <c r="G60" s="9" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
-          <t>Sathya Induri</t>
+          <t>Tony Lam</t>
         </is>
       </c>
       <c r="B61" s="8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C61" s="8" t="inlineStr"/>
       <c r="D61" s="8" t="inlineStr"/>
-      <c r="E61" s="9" t="inlineStr"/>
-      <c r="F61" s="9" t="inlineStr"/>
-      <c r="G61" s="9" t="inlineStr"/>
+      <c r="E61" s="8" t="inlineStr"/>
+      <c r="F61" s="8" t="inlineStr"/>
+      <c r="G61" s="8" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>Shivani Palkar</t>
+          <t>Varadparesh Keni</t>
         </is>
       </c>
       <c r="B62" s="8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C62" s="8" t="inlineStr"/>
       <c r="D62" s="8" t="inlineStr"/>
-      <c r="E62" s="9" t="inlineStr"/>
-      <c r="F62" s="9" t="inlineStr"/>
-      <c r="G62" s="9" t="inlineStr"/>
+      <c r="E62" s="8" t="inlineStr"/>
+      <c r="F62" s="8" t="inlineStr"/>
+      <c r="G62" s="8" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
         <is>
-          <t>Sidhartha Gorajala</t>
+          <t>Varun Bonemone</t>
         </is>
       </c>
       <c r="B63" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C63" s="8" t="inlineStr"/>
-      <c r="D63" s="8" t="inlineStr"/>
-      <c r="E63" s="8" t="inlineStr"/>
+      <c r="D63" s="9" t="inlineStr"/>
+      <c r="E63" s="9" t="inlineStr"/>
       <c r="F63" s="9" t="inlineStr"/>
       <c r="G63" s="9" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
         <is>
-          <t>Srividya Gopala Reddy</t>
+          <t>Vincent Abraham</t>
         </is>
       </c>
       <c r="B64" s="8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C64" s="8" t="inlineStr"/>
       <c r="D64" s="8" t="inlineStr"/>
-      <c r="E64" s="9" t="inlineStr"/>
-      <c r="F64" s="9" t="inlineStr"/>
+      <c r="E64" s="8" t="inlineStr"/>
+      <c r="F64" s="8" t="inlineStr"/>
       <c r="G64" s="9" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
         <is>
-          <t>Tony Lam</t>
+          <t>Yuga Pasupulate</t>
         </is>
       </c>
       <c r="B65" s="8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C65" s="8" t="inlineStr"/>
       <c r="D65" s="8" t="inlineStr"/>
       <c r="E65" s="8" t="inlineStr"/>
       <c r="F65" s="8" t="inlineStr"/>
-      <c r="G65" s="9" t="inlineStr"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="7" t="inlineStr">
-        <is>
-          <t>Trayson Rubio</t>
-        </is>
-      </c>
-      <c r="B66" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C66" s="8" t="inlineStr"/>
-      <c r="D66" s="9" t="inlineStr"/>
-      <c r="E66" s="9" t="inlineStr"/>
-      <c r="F66" s="9" t="inlineStr"/>
-      <c r="G66" s="9" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="7" t="inlineStr">
-        <is>
-          <t>Varadparesh Keni</t>
-        </is>
-      </c>
-      <c r="B67" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="C67" s="8" t="inlineStr"/>
-      <c r="D67" s="8" t="inlineStr"/>
-      <c r="E67" s="8" t="inlineStr"/>
-      <c r="F67" s="8" t="inlineStr"/>
-      <c r="G67" s="8" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="7" t="inlineStr">
-        <is>
-          <t>Vincent Abraham</t>
-        </is>
-      </c>
-      <c r="B68" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="C68" s="8" t="inlineStr"/>
-      <c r="D68" s="8" t="inlineStr"/>
-      <c r="E68" s="8" t="inlineStr"/>
-      <c r="F68" s="8" t="inlineStr"/>
-      <c r="G68" s="9" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="7" t="inlineStr">
-        <is>
-          <t>Yuga Pasupulate</t>
-        </is>
-      </c>
-      <c r="B69" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="C69" s="8" t="inlineStr"/>
-      <c r="D69" s="8" t="inlineStr"/>
-      <c r="E69" s="8" t="inlineStr"/>
-      <c r="F69" s="8" t="inlineStr"/>
-      <c r="G69" s="9" t="inlineStr"/>
+      <c r="G65" s="8" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>